<commit_message>
Calculadora: valores cacheados para que se vea completa al abrirla
Sin los valores cacheados, Felipe abria el archivo y veia celdas en
blanco hasta editar algo. Ahora muestra los numeros de inmediato y
se recalcula solo al tocar cualquier celda.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCN2TjJppTJcfdWR8tc3QB
</commit_message>
<xml_diff>
--- a/descargas/calculadora-pedraza.xlsx
+++ b/descargas/calculadora-pedraza.xlsx
@@ -986,17 +986,17 @@
       </c>
       <c r="D7" s="14" t="n"/>
       <c r="E7" s="16" t="n"/>
-      <c r="F7" s="14">
+      <c r="F7" s="14" t="str">
         <f>IF(E7="","",C7-E7)</f>
         <v/>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="17" t="str">
         <f>IF(E7="","",F7/C7)</f>
         <v/>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="5" t="str">
         <f>IF(E7="","Falta costo",IF(G7&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="8">
@@ -1013,17 +1013,17 @@
       </c>
       <c r="D8" s="14" t="n"/>
       <c r="E8" s="16" t="n"/>
-      <c r="F8" s="14">
+      <c r="F8" s="14" t="str">
         <f>IF(E8="","",C8-E8)</f>
         <v/>
       </c>
-      <c r="G8" s="17">
+      <c r="G8" s="17" t="str">
         <f>IF(E8="","",F8/C8)</f>
         <v/>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="5" t="str">
         <f>IF(E8="","Falta costo",IF(G8&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="9">
@@ -1040,17 +1040,17 @@
       </c>
       <c r="D9" s="14" t="n"/>
       <c r="E9" s="16" t="n"/>
-      <c r="F9" s="14">
+      <c r="F9" s="14" t="str">
         <f>IF(E9="","",C9-E9)</f>
         <v/>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="17" t="str">
         <f>IF(E9="","",F9/C9)</f>
         <v/>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="5" t="str">
         <f>IF(E9="","Falta costo",IF(G9&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="10">
@@ -1069,17 +1069,17 @@
         <v>52990</v>
       </c>
       <c r="E10" s="16" t="n"/>
-      <c r="F10" s="14">
+      <c r="F10" s="14" t="str">
         <f>IF(E10="","",C10-E10)</f>
         <v/>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="17" t="str">
         <f>IF(E10="","",F10/C10)</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="5" t="str">
         <f>IF(E10="","Falta costo",IF(G10&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="11">
@@ -1098,17 +1098,17 @@
         <v>49990</v>
       </c>
       <c r="E11" s="16" t="n"/>
-      <c r="F11" s="14">
+      <c r="F11" s="14" t="str">
         <f>IF(E11="","",C11-E11)</f>
         <v/>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="17" t="str">
         <f>IF(E11="","",F11/C11)</f>
         <v/>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="5" t="str">
         <f>IF(E11="","Falta costo",IF(G11&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="12">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="D12" s="14" t="n"/>
       <c r="E12" s="16" t="n"/>
-      <c r="F12" s="14">
+      <c r="F12" s="14" t="str">
         <f>IF(E12="","",C12-E12)</f>
         <v/>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="17" t="str">
         <f>IF(E12="","",F12/C12)</f>
         <v/>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="5" t="str">
         <f>IF(E12="","Falta costo",IF(G12&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="13">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="D13" s="14" t="n"/>
       <c r="E13" s="16" t="n"/>
-      <c r="F13" s="14">
+      <c r="F13" s="14" t="str">
         <f>IF(E13="","",C13-E13)</f>
         <v/>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="17" t="str">
         <f>IF(E13="","",F13/C13)</f>
         <v/>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="5" t="str">
         <f>IF(E13="","Falta costo",IF(G13&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="14">
@@ -1179,17 +1179,17 @@
       </c>
       <c r="D14" s="14" t="n"/>
       <c r="E14" s="16" t="n"/>
-      <c r="F14" s="14">
+      <c r="F14" s="14" t="str">
         <f>IF(E14="","",C14-E14)</f>
         <v/>
       </c>
-      <c r="G14" s="17">
+      <c r="G14" s="17" t="str">
         <f>IF(E14="","",F14/C14)</f>
         <v/>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="5" t="str">
         <f>IF(E14="","Falta costo",IF(G14&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="15">
@@ -1206,17 +1206,17 @@
       </c>
       <c r="D15" s="14" t="n"/>
       <c r="E15" s="16" t="n"/>
-      <c r="F15" s="14">
+      <c r="F15" s="14" t="str">
         <f>IF(E15="","",C15-E15)</f>
         <v/>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="17" t="str">
         <f>IF(E15="","",F15/C15)</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="5" t="str">
         <f>IF(E15="","Falta costo",IF(G15&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="16">
@@ -1237,15 +1237,15 @@
       </c>
       <c r="F16" s="14">
         <f>IF(E16="","",C16-E16)</f>
-        <v/>
+        <v>22737</v>
       </c>
       <c r="G16" s="17">
         <f>IF(E16="","",F16/C16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="5">
+        <v>0.758152718</v>
+      </c>
+      <c r="H16" s="5" t="str">
         <f>IF(E16="","Falta costo",IF(G16&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>✅ OK</v>
       </c>
     </row>
     <row r="17">
@@ -1262,17 +1262,17 @@
       </c>
       <c r="D17" s="14" t="n"/>
       <c r="E17" s="16" t="n"/>
-      <c r="F17" s="14">
+      <c r="F17" s="14" t="str">
         <f>IF(E17="","",C17-E17)</f>
         <v/>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="17" t="str">
         <f>IF(E17="","",F17/C17)</f>
         <v/>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="5" t="str">
         <f>IF(E17="","Falta costo",IF(G17&lt;0.6,"⚠ BAJO 60%","✅ OK"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
@@ -1395,9 +1395,9 @@
       </c>
       <c r="B7" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A7,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C7" s="14">
+        <v>32990</v>
+      </c>
+      <c r="C7" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A7,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1406,19 +1406,19 @@
       </c>
       <c r="E7" s="15">
         <f>IF(B7="","",B7*(1-D7))</f>
-        <v/>
-      </c>
-      <c r="F7" s="14">
+        <v>29691</v>
+      </c>
+      <c r="F7" s="14" t="str">
         <f>IF(OR(B7="",C7="",C7=0),"",E7-C7)</f>
         <v/>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="17" t="str">
         <f>IF(F7="","",IF(E7=0,"",F7/E7))</f>
         <v/>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="5" t="str">
         <f>IF(F7="","Falta costo",IF(G7&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="8">
@@ -1429,9 +1429,9 @@
       </c>
       <c r="B8" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A8,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C8" s="14">
+        <v>9990</v>
+      </c>
+      <c r="C8" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A8,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1440,19 +1440,19 @@
       </c>
       <c r="E8" s="15">
         <f>IF(B8="","",B8*(1-D8))</f>
-        <v/>
-      </c>
-      <c r="F8" s="14">
+        <v>8991</v>
+      </c>
+      <c r="F8" s="14" t="str">
         <f>IF(OR(B8="",C8="",C8=0),"",E8-C8)</f>
         <v/>
       </c>
-      <c r="G8" s="17">
+      <c r="G8" s="17" t="str">
         <f>IF(F8="","",IF(E8=0,"",F8/E8))</f>
         <v/>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="5" t="str">
         <f>IF(F8="","Falta costo",IF(G8&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="9">
@@ -1463,9 +1463,9 @@
       </c>
       <c r="B9" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A9,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C9" s="14">
+        <v>22990</v>
+      </c>
+      <c r="C9" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A9,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1474,19 +1474,19 @@
       </c>
       <c r="E9" s="15">
         <f>IF(B9="","",B9*(1-D9))</f>
-        <v/>
-      </c>
-      <c r="F9" s="14">
+        <v>20691</v>
+      </c>
+      <c r="F9" s="14" t="str">
         <f>IF(OR(B9="",C9="",C9=0),"",E9-C9)</f>
         <v/>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="17" t="str">
         <f>IF(F9="","",IF(E9=0,"",F9/E9))</f>
         <v/>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="5" t="str">
         <f>IF(F9="","Falta costo",IF(G9&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="10">
@@ -1497,9 +1497,9 @@
       </c>
       <c r="B10" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A10,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C10" s="14">
+        <v>42990</v>
+      </c>
+      <c r="C10" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A10,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1508,19 +1508,19 @@
       </c>
       <c r="E10" s="15">
         <f>IF(B10="","",B10*(1-D10))</f>
-        <v/>
-      </c>
-      <c r="F10" s="14">
+        <v>38691</v>
+      </c>
+      <c r="F10" s="14" t="str">
         <f>IF(OR(B10="",C10="",C10=0),"",E10-C10)</f>
         <v/>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="17" t="str">
         <f>IF(F10="","",IF(E10=0,"",F10/E10))</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="5" t="str">
         <f>IF(F10="","Falta costo",IF(G10&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="11">
@@ -1531,9 +1531,9 @@
       </c>
       <c r="B11" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A11,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C11" s="14">
+        <v>32990</v>
+      </c>
+      <c r="C11" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A11,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1542,19 +1542,19 @@
       </c>
       <c r="E11" s="15">
         <f>IF(B11="","",B11*(1-D11))</f>
-        <v/>
-      </c>
-      <c r="F11" s="14">
+        <v>29691</v>
+      </c>
+      <c r="F11" s="14" t="str">
         <f>IF(OR(B11="",C11="",C11=0),"",E11-C11)</f>
         <v/>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="17" t="str">
         <f>IF(F11="","",IF(E11=0,"",F11/E11))</f>
         <v/>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="5" t="str">
         <f>IF(F11="","Falta costo",IF(G11&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="12">
@@ -1565,9 +1565,9 @@
       </c>
       <c r="B12" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A12,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C12" s="14">
+        <v>18990</v>
+      </c>
+      <c r="C12" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A12,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1576,19 +1576,19 @@
       </c>
       <c r="E12" s="15">
         <f>IF(B12="","",B12*(1-D12))</f>
-        <v/>
-      </c>
-      <c r="F12" s="14">
+        <v>17091</v>
+      </c>
+      <c r="F12" s="14" t="str">
         <f>IF(OR(B12="",C12="",C12=0),"",E12-C12)</f>
         <v/>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="17" t="str">
         <f>IF(F12="","",IF(E12=0,"",F12/E12))</f>
         <v/>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="5" t="str">
         <f>IF(F12="","Falta costo",IF(G12&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="13">
@@ -1599,9 +1599,9 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A13,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C13" s="14">
+        <v>9990</v>
+      </c>
+      <c r="C13" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A13,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1610,19 +1610,19 @@
       </c>
       <c r="E13" s="15">
         <f>IF(B13="","",B13*(1-D13))</f>
-        <v/>
-      </c>
-      <c r="F13" s="14">
+        <v>8991</v>
+      </c>
+      <c r="F13" s="14" t="str">
         <f>IF(OR(B13="",C13="",C13=0),"",E13-C13)</f>
         <v/>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="17" t="str">
         <f>IF(F13="","",IF(E13=0,"",F13/E13))</f>
         <v/>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="5" t="str">
         <f>IF(F13="","Falta costo",IF(G13&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="14">
@@ -1633,9 +1633,9 @@
       </c>
       <c r="B14" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A14,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C14" s="14">
+        <v>7990</v>
+      </c>
+      <c r="C14" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A14,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1644,19 +1644,19 @@
       </c>
       <c r="E14" s="15">
         <f>IF(B14="","",B14*(1-D14))</f>
-        <v/>
-      </c>
-      <c r="F14" s="14">
+        <v>7191</v>
+      </c>
+      <c r="F14" s="14" t="str">
         <f>IF(OR(B14="",C14="",C14=0),"",E14-C14)</f>
         <v/>
       </c>
-      <c r="G14" s="17">
+      <c r="G14" s="17" t="str">
         <f>IF(F14="","",IF(E14=0,"",F14/E14))</f>
         <v/>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="5" t="str">
         <f>IF(F14="","Falta costo",IF(G14&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="15">
@@ -1667,9 +1667,9 @@
       </c>
       <c r="B15" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A15,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C15" s="14">
+        <v>11990</v>
+      </c>
+      <c r="C15" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A15,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1678,19 +1678,19 @@
       </c>
       <c r="E15" s="15">
         <f>IF(B15="","",B15*(1-D15))</f>
-        <v/>
-      </c>
-      <c r="F15" s="14">
+        <v>10791</v>
+      </c>
+      <c r="F15" s="14" t="str">
         <f>IF(OR(B15="",C15="",C15=0),"",E15-C15)</f>
         <v/>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="17" t="str">
         <f>IF(F15="","",IF(E15=0,"",F15/E15))</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="5" t="str">
         <f>IF(F15="","Falta costo",IF(G15&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="16">
@@ -1701,30 +1701,30 @@
       </c>
       <c r="B16" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A16,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
+        <v>29990</v>
       </c>
       <c r="C16" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A16,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
+        <v>7253</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>0.1</v>
       </c>
       <c r="E16" s="15">
         <f>IF(B16="","",B16*(1-D16))</f>
-        <v/>
+        <v>26991</v>
       </c>
       <c r="F16" s="14">
         <f>IF(OR(B16="",C16="",C16=0),"",E16-C16)</f>
-        <v/>
+        <v>19738</v>
       </c>
       <c r="G16" s="17">
         <f>IF(F16="","",IF(E16=0,"",F16/E16))</f>
-        <v/>
-      </c>
-      <c r="H16" s="5">
+        <v>0.731280797</v>
+      </c>
+      <c r="H16" s="5" t="str">
         <f>IF(F16="","Falta costo",IF(G16&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>✅ OK, sobre el piso</v>
       </c>
     </row>
     <row r="17">
@@ -1735,9 +1735,9 @@
       </c>
       <c r="B17" s="14">
         <f>IFERROR(INDEX('Escala de valor'!$C$7:$C$17,MATCH(A17,'Escala de valor'!$A$7:$A$17,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C17" s="14">
+        <v>17990</v>
+      </c>
+      <c r="C17" s="14" t="str">
         <f>IFERROR(INDEX('Escala de valor'!$E$7:$E$17,MATCH(A17,'Escala de valor'!$A$7:$A$17,0)),"")</f>
         <v/>
       </c>
@@ -1746,19 +1746,19 @@
       </c>
       <c r="E17" s="15">
         <f>IF(B17="","",B17*(1-D17))</f>
-        <v/>
-      </c>
-      <c r="F17" s="14">
+        <v>16191</v>
+      </c>
+      <c r="F17" s="14" t="str">
         <f>IF(OR(B17="",C17="",C17=0),"",E17-C17)</f>
         <v/>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="17" t="str">
         <f>IF(F17="","",IF(E17=0,"",F17/E17))</f>
         <v/>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="5" t="str">
         <f>IF(F17="","Falta costo",IF(G17&lt;0.6,"⚠ CAE BAJO 60%","✅ OK, sobre el piso"))</f>
-        <v/>
+        <v>Falta costo</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
@@ -1885,14 +1885,14 @@
       </c>
       <c r="E6" s="22">
         <f>SUM(B6:D6)</f>
-        <v/>
+        <v>1678</v>
       </c>
       <c r="F6" s="21" t="n">
         <v>1290</v>
       </c>
       <c r="G6" s="22">
         <f>E6-F6</f>
-        <v/>
+        <v>388</v>
       </c>
     </row>
     <row r="7">
@@ -1912,14 +1912,14 @@
       </c>
       <c r="E7" s="22">
         <f>SUM(B7:D7)</f>
-        <v/>
+        <v>2157</v>
       </c>
       <c r="F7" s="21" t="n">
         <v>1290</v>
       </c>
       <c r="G7" s="22">
         <f>E7-F7</f>
-        <v/>
+        <v>867</v>
       </c>
     </row>
     <row r="8">
@@ -1939,14 +1939,14 @@
       </c>
       <c r="E8" s="22">
         <f>SUM(B8:D8)</f>
-        <v/>
+        <v>2519</v>
       </c>
       <c r="F8" s="21" t="n">
         <v>1290</v>
       </c>
       <c r="G8" s="22">
         <f>E8-F8</f>
-        <v/>
+        <v>1229</v>
       </c>
     </row>
     <row r="9">
@@ -1966,14 +1966,14 @@
       </c>
       <c r="E9" s="22">
         <f>SUM(B9:D9)</f>
-        <v/>
+        <v>2859</v>
       </c>
       <c r="F9" s="21" t="n">
         <v>1290</v>
       </c>
       <c r="G9" s="22">
         <f>E9-F9</f>
-        <v/>
+        <v>1569</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
@@ -2015,9 +2015,9 @@
       <c r="F14" s="20" t="n">
         <v>0.16</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="8" t="str">
         <f>IF(B14+D14+F14&lt;&gt;1,"⚠ no suma 100%","✅ 100%")</f>
-        <v/>
+        <v>✅ 100%</v>
       </c>
     </row>
     <row r="16">
@@ -2055,19 +2055,19 @@
       </c>
       <c r="B17" s="24">
         <f>E6</f>
-        <v/>
+        <v>1678</v>
       </c>
       <c r="C17" s="24">
         <f>$B17*$B$14</f>
-        <v/>
+        <v>788.66</v>
       </c>
       <c r="D17" s="24">
         <f>$B17*$D$14</f>
-        <v/>
+        <v>620.86</v>
       </c>
       <c r="E17" s="24">
         <f>$B17*$F$14</f>
-        <v/>
+        <v>268.48</v>
       </c>
     </row>
     <row r="18">
@@ -2078,19 +2078,19 @@
       </c>
       <c r="B18" s="24">
         <f>E7</f>
-        <v/>
+        <v>2157</v>
       </c>
       <c r="C18" s="24">
         <f>$B18*$B$14</f>
-        <v/>
+        <v>1013.79</v>
       </c>
       <c r="D18" s="24">
         <f>$B18*$D$14</f>
-        <v/>
+        <v>798.09</v>
       </c>
       <c r="E18" s="24">
         <f>$B18*$F$14</f>
-        <v/>
+        <v>345.12</v>
       </c>
     </row>
     <row r="19">
@@ -2101,19 +2101,19 @@
       </c>
       <c r="B19" s="24">
         <f>E8</f>
-        <v/>
+        <v>2519</v>
       </c>
       <c r="C19" s="24">
         <f>$B19*$B$14</f>
-        <v/>
+        <v>1183.93</v>
       </c>
       <c r="D19" s="24">
         <f>$B19*$D$14</f>
-        <v/>
+        <v>932.03</v>
       </c>
       <c r="E19" s="24">
         <f>$B19*$F$14</f>
-        <v/>
+        <v>403.04</v>
       </c>
     </row>
     <row r="20">
@@ -2124,19 +2124,19 @@
       </c>
       <c r="B20" s="24">
         <f>E9</f>
-        <v/>
+        <v>2859</v>
       </c>
       <c r="C20" s="24">
         <f>$B20*$B$14</f>
-        <v/>
+        <v>1343.73</v>
       </c>
       <c r="D20" s="24">
         <f>$B20*$D$14</f>
-        <v/>
+        <v>1057.83</v>
       </c>
       <c r="E20" s="24">
         <f>$B20*$F$14</f>
-        <v/>
+        <v>457.44</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
@@ -2279,14 +2279,14 @@
       </c>
       <c r="C12" s="24">
         <f>$B$5*B12</f>
-        <v/>
+        <v>940</v>
       </c>
       <c r="D12" s="26" t="n">
         <v>4.8</v>
       </c>
       <c r="E12" s="27">
         <f>C12*D12</f>
-        <v/>
+        <v>4512</v>
       </c>
     </row>
     <row r="13">
@@ -2300,14 +2300,14 @@
       </c>
       <c r="C13" s="24">
         <f>$B$5*B13</f>
-        <v/>
+        <v>740</v>
       </c>
       <c r="D13" s="26" t="n">
         <v>5.8</v>
       </c>
       <c r="E13" s="27">
         <f>C13*D13</f>
-        <v/>
+        <v>4292</v>
       </c>
     </row>
     <row r="14">
@@ -2321,14 +2321,14 @@
       </c>
       <c r="C14" s="24">
         <f>$B$5*B14</f>
-        <v/>
+        <v>320</v>
       </c>
       <c r="D14" s="26" t="n">
         <v>6.48</v>
       </c>
       <c r="E14" s="27">
         <f>C14*D14</f>
-        <v/>
+        <v>2073.6</v>
       </c>
     </row>
     <row r="15">
@@ -2339,21 +2339,21 @@
       </c>
       <c r="B15" s="28">
         <f>SUM(B12:B14)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="C15" s="22">
         <f>SUM(C12:C14)</f>
-        <v/>
+        <v>2000</v>
       </c>
       <c r="E15" s="29">
         <f>SUM(E12:E14)</f>
-        <v/>
+        <v>10877.6</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8">
+      <c r="A16" s="8" t="str">
         <f>IF(B15&lt;&gt;1,"⚠ el reparto no suma 100%","✅ el reparto suma 100%")</f>
-        <v/>
+        <v>✅ el reparto suma 100%</v>
       </c>
     </row>
     <row r="18">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B20" s="29">
         <f>E15</f>
-        <v/>
+        <v>10877.6</v>
       </c>
     </row>
     <row r="21">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B21" s="15">
         <f>B20*B6</f>
-        <v/>
+        <v>10333720</v>
       </c>
     </row>
     <row r="22">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="B22" s="27">
         <f>B20*B7</f>
-        <v/>
+        <v>3263.28</v>
       </c>
     </row>
     <row r="23">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B23" s="15">
         <f>B22*B6</f>
-        <v/>
+        <v>3100116</v>
       </c>
     </row>
     <row r="24">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="B24" s="14">
         <f>B21-B23</f>
-        <v/>
+        <v>7233604</v>
       </c>
     </row>
     <row r="25">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="B25" s="15">
         <f>B5*B8</f>
-        <v/>
+        <v>14506000</v>
       </c>
     </row>
     <row r="26">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="B26" s="14">
         <f>B25-B21</f>
-        <v/>
+        <v>4172280</v>
       </c>
     </row>
     <row r="28">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B29" s="31">
         <f>B23/B28</f>
-        <v/>
+        <v>2.656191952</v>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1">
@@ -2576,18 +2576,18 @@
       </c>
       <c r="C7" s="32">
         <f>B7/18</f>
-        <v/>
+        <v>102.055555556</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="33">
         <f>IF(D7="","",IF(C7=0,"",D7/C7))</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="str">
         <f>IF(E7="","Falta stock",IF(E7&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>🔴 BAJO 2 MESES</v>
       </c>
     </row>
     <row r="8">
@@ -2601,16 +2601,16 @@
       </c>
       <c r="C8" s="32">
         <f>B8/18</f>
-        <v/>
+        <v>37.888888889</v>
       </c>
       <c r="D8" s="21" t="n"/>
-      <c r="E8" s="33">
+      <c r="E8" s="33" t="str">
         <f>IF(D8="","",IF(C8=0,"",D8/C8))</f>
         <v/>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="5" t="str">
         <f>IF(E8="","Falta stock",IF(E8&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="9">
@@ -2624,16 +2624,16 @@
       </c>
       <c r="C9" s="32">
         <f>B9/18</f>
-        <v/>
+        <v>36.888888889</v>
       </c>
       <c r="D9" s="21" t="n"/>
-      <c r="E9" s="33">
+      <c r="E9" s="33" t="str">
         <f>IF(D9="","",IF(C9=0,"",D9/C9))</f>
         <v/>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="5" t="str">
         <f>IF(E9="","Falta stock",IF(E9&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="10">
@@ -2647,16 +2647,16 @@
       </c>
       <c r="C10" s="32">
         <f>B10/18</f>
-        <v/>
+        <v>31.444444444</v>
       </c>
       <c r="D10" s="21" t="n"/>
-      <c r="E10" s="33">
+      <c r="E10" s="33" t="str">
         <f>IF(D10="","",IF(C10=0,"",D10/C10))</f>
         <v/>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="5" t="str">
         <f>IF(E10="","Falta stock",IF(E10&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="11">
@@ -2670,16 +2670,16 @@
       </c>
       <c r="C11" s="32">
         <f>B11/18</f>
-        <v/>
+        <v>17.777777778</v>
       </c>
       <c r="D11" s="21" t="n"/>
-      <c r="E11" s="33">
+      <c r="E11" s="33" t="str">
         <f>IF(D11="","",IF(C11=0,"",D11/C11))</f>
         <v/>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="5" t="str">
         <f>IF(E11="","Falta stock",IF(E11&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="12">
@@ -2693,16 +2693,16 @@
       </c>
       <c r="C12" s="32">
         <f>B12/18</f>
-        <v/>
+        <v>16.555555556</v>
       </c>
       <c r="D12" s="21" t="n"/>
-      <c r="E12" s="33">
+      <c r="E12" s="33" t="str">
         <f>IF(D12="","",IF(C12=0,"",D12/C12))</f>
         <v/>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="5" t="str">
         <f>IF(E12="","Falta stock",IF(E12&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="13">
@@ -2716,16 +2716,16 @@
       </c>
       <c r="C13" s="32">
         <f>B13/18</f>
-        <v/>
+        <v>14.888888889</v>
       </c>
       <c r="D13" s="21" t="n"/>
-      <c r="E13" s="33">
+      <c r="E13" s="33" t="str">
         <f>IF(D13="","",IF(C13=0,"",D13/C13))</f>
         <v/>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="5" t="str">
         <f>IF(E13="","Falta stock",IF(E13&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="14">
@@ -2739,16 +2739,16 @@
       </c>
       <c r="C14" s="32">
         <f>B14/18</f>
-        <v/>
+        <v>9.111111111</v>
       </c>
       <c r="D14" s="21" t="n"/>
-      <c r="E14" s="33">
+      <c r="E14" s="33" t="str">
         <f>IF(D14="","",IF(C14=0,"",D14/C14))</f>
         <v/>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="5" t="str">
         <f>IF(E14="","Falta stock",IF(E14&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="15">
@@ -2762,16 +2762,16 @@
       </c>
       <c r="C15" s="32">
         <f>B15/18</f>
-        <v/>
+        <v>8.555555556</v>
       </c>
       <c r="D15" s="21" t="n"/>
-      <c r="E15" s="33">
+      <c r="E15" s="33" t="str">
         <f>IF(D15="","",IF(C15=0,"",D15/C15))</f>
         <v/>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="5" t="str">
         <f>IF(E15="","Falta stock",IF(E15&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="16">
@@ -2785,16 +2785,16 @@
       </c>
       <c r="C16" s="32">
         <f>B16/18</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="D16" s="21" t="n"/>
-      <c r="E16" s="33">
+      <c r="E16" s="33" t="str">
         <f>IF(D16="","",IF(C16=0,"",D16/C16))</f>
         <v/>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="5" t="str">
         <f>IF(E16="","Falta stock",IF(E16&lt;2,"🔴 BAJO 2 MESES","🟢 OK"))</f>
-        <v/>
+        <v>Falta stock</v>
       </c>
     </row>
     <row r="17">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B17" s="22">
         <f>SUM(B7:B16)</f>
-        <v/>
+        <v>5097</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">

</xml_diff>